<commit_message>
entrega 2 finalizada e atualização dos dados (04/2020 - 03/2025).
</commit_message>
<xml_diff>
--- a/entregas/cronograma.xlsx
+++ b/entregas/cronograma.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Cronograma_Gantt" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="cronograma" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="67">
   <si>
     <t>Nome da Atividade</t>
   </si>
@@ -73,27 +73,33 @@
     <t>20/08/26</t>
   </si>
   <si>
+    <t>todos</t>
+  </si>
+  <si>
     <t>-</t>
   </si>
   <si>
+    <t>Finalizado</t>
+  </si>
+  <si>
+    <t>Objetivos e Cronograma (Entrega 2)</t>
+  </si>
+  <si>
+    <t>Definição do título, objetivos e organização detalhada do cronograma.</t>
+  </si>
+  <si>
+    <t>21/08/26</t>
+  </si>
+  <si>
+    <t>10/09/26</t>
+  </si>
+  <si>
+    <t>Entrega 1</t>
+  </si>
+  <si>
     <t>A fazer</t>
   </si>
   <si>
-    <t>Objetivos e Cronograma (Entrega 2)</t>
-  </si>
-  <si>
-    <t>Definição do título, objetivos e organização detalhada do cronograma.</t>
-  </si>
-  <si>
-    <t>21/08/26</t>
-  </si>
-  <si>
-    <t>10/09/26</t>
-  </si>
-  <si>
-    <t>Entrega 1</t>
-  </si>
-  <si>
     <t>Estudo Teórico das Metodologias</t>
   </si>
   <si>
@@ -101,6 +107,9 @@
   </si>
   <si>
     <t>15/09/26</t>
+  </si>
+  <si>
+    <t>Markowitz e 1/N: Phillip; Shannon Entropy: Eduardo; Tsallis Entropy: Waleska; Weighted Shannon Entropy: Kauã</t>
   </si>
   <si>
     <t>Implementação das Metodologias</t>
@@ -296,7 +305,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -313,6 +322,9 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -727,9 +739,11 @@
       <c r="D2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="4"/>
+      <c r="E2" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="F2" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="6"/>
@@ -741,25 +755,27 @@
       <c r="N2" s="6"/>
       <c r="O2" s="6"/>
       <c r="P2" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="47.25" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E3" s="4"/>
+        <v>26</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="F3" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G3" s="7"/>
       <c r="H3" s="5"/>
@@ -771,25 +787,27 @@
       <c r="N3" s="7"/>
       <c r="O3" s="7"/>
       <c r="P3" s="6" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" ht="112.5" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="G4" s="6"/>
       <c r="H4" s="5"/>
@@ -801,25 +819,27 @@
       <c r="N4" s="6"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="39.75" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="4"/>
+        <v>36</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="F5" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="G5" s="7"/>
       <c r="H5" s="5"/>
@@ -831,25 +851,27 @@
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
       <c r="P5" s="6" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="43.5" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="E6" s="4"/>
+        <v>41</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="F6" s="4" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -861,25 +883,27 @@
       <c r="N6" s="6"/>
       <c r="O6" s="6"/>
       <c r="P6" s="6" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="40.5" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E7" s="4"/>
+        <v>46</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="F7" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
@@ -891,25 +915,27 @@
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
       <c r="P7" s="6" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="40.5" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>42</v>
-      </c>
       <c r="D8" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E8" s="4"/>
+        <v>50</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="F8" s="4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
@@ -921,25 +947,27 @@
       <c r="N8" s="6"/>
       <c r="O8" s="6"/>
       <c r="P8" s="6" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="39" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="E9" s="4"/>
+        <v>55</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="F9" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
@@ -951,25 +979,27 @@
       <c r="N9" s="5"/>
       <c r="O9" s="7"/>
       <c r="P9" s="6" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" ht="33" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E10" s="4"/>
+        <v>60</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="F10" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
@@ -981,25 +1011,27 @@
       <c r="N10" s="5"/>
       <c r="O10" s="6"/>
       <c r="P10" s="6" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" ht="52.5" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E11" s="4"/>
+        <v>65</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="F11" s="4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
@@ -1011,7 +1043,7 @@
       <c r="N11" s="5"/>
       <c r="O11" s="5"/>
       <c r="P11" s="6" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>